<commit_message>
Update KPI tooltip text
</commit_message>
<xml_diff>
--- a/output/qa/Tidyed_Data_v2.xlsx
+++ b/output/qa/Tidyed_Data_v2.xlsx
@@ -1012,13 +1012,13 @@
         <v>1</v>
       </c>
       <c r="AB3" t="n">
+        <v>100</v>
+      </c>
+      <c r="AC3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD3" t="n">
         <v>99.12280699999999</v>
-      </c>
-      <c r="AC3" t="n">
-        <v>1</v>
-      </c>
-      <c r="AD3" t="n">
-        <v>100</v>
       </c>
       <c r="AE3" t="n">
         <v>0</v>
@@ -1424,13 +1424,13 @@
         <v>0</v>
       </c>
       <c r="AB5" t="n">
-        <v>100</v>
+        <v>96.791444</v>
       </c>
       <c r="AC5" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AD5" t="n">
-        <v>96.791444</v>
+        <v>100</v>
       </c>
       <c r="AE5" t="n">
         <v>2</v>
@@ -1818,13 +1818,13 @@
         <v>3</v>
       </c>
       <c r="AB7" t="n">
+        <v>100</v>
+      </c>
+      <c r="AC7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD7" t="n">
         <v>84.210526</v>
-      </c>
-      <c r="AC7" t="n">
-        <v>3</v>
-      </c>
-      <c r="AD7" t="n">
-        <v>100</v>
       </c>
       <c r="AE7" t="n">
         <v>2</v>
@@ -2224,13 +2224,13 @@
         <v>2</v>
       </c>
       <c r="AB9" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AC9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AD9" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="AE9" t="n">
         <v>0</v>
@@ -2434,13 +2434,13 @@
         <v>3</v>
       </c>
       <c r="AB10" t="n">
+        <v>97.61904800000001</v>
+      </c>
+      <c r="AC10" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD10" t="n">
         <v>92.85714299999999</v>
-      </c>
-      <c r="AC10" t="n">
-        <v>3</v>
-      </c>
-      <c r="AD10" t="n">
-        <v>97.61904800000001</v>
       </c>
       <c r="AE10" t="n">
         <v>0</v>
@@ -2646,13 +2646,13 @@
         <v>3</v>
       </c>
       <c r="AB11" t="n">
+        <v>100</v>
+      </c>
+      <c r="AC11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD11" t="n">
         <v>97.39130400000001</v>
-      </c>
-      <c r="AC11" t="n">
-        <v>3</v>
-      </c>
-      <c r="AD11" t="n">
-        <v>100</v>
       </c>
       <c r="AE11" t="n">
         <v>1</v>
@@ -2856,13 +2856,13 @@
         <v>1</v>
       </c>
       <c r="AB12" t="n">
+        <v>97.252747</v>
+      </c>
+      <c r="AC12" t="n">
+        <v>5</v>
+      </c>
+      <c r="AD12" t="n">
         <v>99.450549</v>
-      </c>
-      <c r="AC12" t="n">
-        <v>1</v>
-      </c>
-      <c r="AD12" t="n">
-        <v>97.252747</v>
       </c>
       <c r="AE12" t="n">
         <v/>
@@ -3060,13 +3060,13 @@
         <v>47</v>
       </c>
       <c r="AB13" t="n">
+        <v>99.880168</v>
+      </c>
+      <c r="AC13" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD13" t="n">
         <v>97.183942</v>
-      </c>
-      <c r="AC13" t="n">
-        <v>47</v>
-      </c>
-      <c r="AD13" t="n">
-        <v>99.880168</v>
       </c>
       <c r="AE13" t="n">
         <v>0</v>
@@ -5715,13 +5715,13 @@
         <v>41</v>
       </c>
       <c r="AB26" t="n">
+        <v>94.385593</v>
+      </c>
+      <c r="AC26" t="n">
+        <v>53</v>
+      </c>
+      <c r="AD26" t="n">
         <v>95.65678</v>
-      </c>
-      <c r="AC26" t="n">
-        <v>41</v>
-      </c>
-      <c r="AD26" t="n">
-        <v>94.385593</v>
       </c>
       <c r="AE26" t="n">
         <v>34</v>
@@ -5924,13 +5924,13 @@
         <v>1</v>
       </c>
       <c r="AB27" t="n">
+        <v>100</v>
+      </c>
+      <c r="AC27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD27" t="n">
         <v>91.666667</v>
-      </c>
-      <c r="AC27" t="n">
-        <v>1</v>
-      </c>
-      <c r="AD27" t="n">
-        <v>100</v>
       </c>
       <c r="AE27" t="n">
         <v>0</v>
@@ -6505,13 +6505,13 @@
         <v>8</v>
       </c>
       <c r="AB30" t="n">
+        <v>94.38202200000001</v>
+      </c>
+      <c r="AC30" t="n">
+        <v>5</v>
+      </c>
+      <c r="AD30" t="n">
         <v>91.011236</v>
-      </c>
-      <c r="AC30" t="n">
-        <v>8</v>
-      </c>
-      <c r="AD30" t="n">
-        <v>94.38202200000001</v>
       </c>
       <c r="AE30" t="n">
         <v>0</v>
@@ -6910,13 +6910,13 @@
         <v>1</v>
       </c>
       <c r="AB32" t="n">
+        <v>100</v>
+      </c>
+      <c r="AC32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD32" t="n">
         <v>93.75</v>
-      </c>
-      <c r="AC32" t="n">
-        <v>1</v>
-      </c>
-      <c r="AD32" t="n">
-        <v>100</v>
       </c>
       <c r="AE32" t="n">
         <v>0</v>
@@ -7693,13 +7693,13 @@
         <v>5</v>
       </c>
       <c r="AB36" t="n">
+        <v>100</v>
+      </c>
+      <c r="AC36" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD36" t="n">
         <v>95.614035</v>
-      </c>
-      <c r="AC36" t="n">
-        <v>5</v>
-      </c>
-      <c r="AD36" t="n">
-        <v>100</v>
       </c>
       <c r="AE36" t="n">
         <v>0</v>
@@ -8502,13 +8502,13 @@
         <v>2</v>
       </c>
       <c r="AB40" t="n">
+        <v>100</v>
+      </c>
+      <c r="AC40" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD40" t="n">
         <v>89.47368400000001</v>
-      </c>
-      <c r="AC40" t="n">
-        <v>2</v>
-      </c>
-      <c r="AD40" t="n">
-        <v>100</v>
       </c>
       <c r="AE40" t="n">
         <v>0</v>
@@ -8909,13 +8909,13 @@
         <v>2</v>
       </c>
       <c r="AB42" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AC42" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AD42" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="AE42" t="n">
         <v>0</v>
@@ -9101,13 +9101,13 @@
         <v>2</v>
       </c>
       <c r="AB43" t="n">
+        <v>100</v>
+      </c>
+      <c r="AC43" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD43" t="n">
         <v>97.058824</v>
-      </c>
-      <c r="AC43" t="n">
-        <v>2</v>
-      </c>
-      <c r="AD43" t="n">
-        <v>100</v>
       </c>
       <c r="AE43" t="n">
         <v>2</v>
@@ -9738,13 +9738,13 @@
         <v>58</v>
       </c>
       <c r="AB46" t="n">
+        <v>99.93831</v>
+      </c>
+      <c r="AC46" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD46" t="n">
         <v>96.42196199999999</v>
-      </c>
-      <c r="AC46" t="n">
-        <v>58</v>
-      </c>
-      <c r="AD46" t="n">
-        <v>99.93831</v>
       </c>
       <c r="AE46" t="n">
         <v>0</v>
@@ -12380,13 +12380,13 @@
         <v>45</v>
       </c>
       <c r="AB59" t="n">
+        <v>100</v>
+      </c>
+      <c r="AC59" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD59" t="n">
         <v>95.227996</v>
-      </c>
-      <c r="AC59" t="n">
-        <v>45</v>
-      </c>
-      <c r="AD59" t="n">
-        <v>100</v>
       </c>
       <c r="AE59" t="n">
         <v>23</v>
@@ -12589,13 +12589,13 @@
         <v>1</v>
       </c>
       <c r="AB60" t="n">
+        <v>100</v>
+      </c>
+      <c r="AC60" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD60" t="n">
         <v>93.75</v>
-      </c>
-      <c r="AC60" t="n">
-        <v>1</v>
-      </c>
-      <c r="AD60" t="n">
-        <v>100</v>
       </c>
       <c r="AE60" t="n">
         <v>0</v>

</xml_diff>